<commit_message>
Grava valor em cache das formulas na planilha gerada
openpyxl salva a formula sem valor calculado, entao qualquer leitor que nao
recalcula (pandas, previa de e-mail, visualizador de celular) mostrava a
celula vazia. Agora o gerador injeta o <v> de cada formula direto no XML,
como o proprio Excel salvaria, e marca fullCalcOnLoad para o Excel/Calc
recalcular tudo na abertura. As formulas seguem intactas.

Inclui a planilha gerada com as 10 pecas da Revenda 1 (280 pecas no total).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjicBvHCdScDry7mP1iFsP
</commit_message>
<xml_diff>
--- a/Estoque_Minimo_Revenda1_2026-08-27.xlsx
+++ b/Estoque_Minimo_Revenda1_2026-08-27.xlsx
@@ -554,7 +554,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -677,15 +677,15 @@
       </c>
       <c r="G9" s="9">
         <f>MAX(F9-E9,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H9" s="10">
         <f>MAX(G9,ROUND(F9*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I9" s="6">
+        <v>130</v>
+      </c>
+      <c r="I9" s="6" t="str">
         <f>IF(E9&lt;=0,"Crítico",IF(E9&lt;F9,"Abaixo do Mínimo",IF(E9=F9,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="10">
@@ -709,15 +709,15 @@
       </c>
       <c r="G10" s="9">
         <f>MAX(F10-E10,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H10" s="10">
         <f>MAX(G10,ROUND(F10*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I10" s="6">
+        <v>60</v>
+      </c>
+      <c r="I10" s="6" t="str">
         <f>IF(E10&lt;=0,"Crítico",IF(E10&lt;F10,"Abaixo do Mínimo",IF(E10=F10,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="11">
@@ -741,15 +741,15 @@
       </c>
       <c r="G11" s="9">
         <f>MAX(F11-E11,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H11" s="10">
         <f>MAX(G11,ROUND(F11*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I11" s="6">
+        <v>50</v>
+      </c>
+      <c r="I11" s="6" t="str">
         <f>IF(E11&lt;=0,"Crítico",IF(E11&lt;F11,"Abaixo do Mínimo",IF(E11=F11,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="12">
@@ -773,15 +773,15 @@
       </c>
       <c r="G12" s="9">
         <f>MAX(F12-E12,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H12" s="10">
         <f>MAX(G12,ROUND(F12*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I12" s="6">
+        <v>15</v>
+      </c>
+      <c r="I12" s="6" t="str">
         <f>IF(E12&lt;=0,"Crítico",IF(E12&lt;F12,"Abaixo do Mínimo",IF(E12=F12,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="13">
@@ -805,15 +805,15 @@
       </c>
       <c r="G13" s="9">
         <f>MAX(F13-E13,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H13" s="10">
         <f>MAX(G13,ROUND(F13*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I13" s="6">
+        <v>15</v>
+      </c>
+      <c r="I13" s="6" t="str">
         <f>IF(E13&lt;=0,"Crítico",IF(E13&lt;F13,"Abaixo do Mínimo",IF(E13=F13,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="14">
@@ -837,15 +837,15 @@
       </c>
       <c r="G14" s="9">
         <f>MAX(F14-E14,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H14" s="10">
         <f>MAX(G14,ROUND(F14*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I14" s="6">
+        <v>4</v>
+      </c>
+      <c r="I14" s="6" t="str">
         <f>IF(E14&lt;=0,"Crítico",IF(E14&lt;F14,"Abaixo do Mínimo",IF(E14=F14,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="15">
@@ -869,15 +869,15 @@
       </c>
       <c r="G15" s="9">
         <f>MAX(F15-E15,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H15" s="10">
         <f>MAX(G15,ROUND(F15*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I15" s="6">
+        <v>2</v>
+      </c>
+      <c r="I15" s="6" t="str">
         <f>IF(E15&lt;=0,"Crítico",IF(E15&lt;F15,"Abaixo do Mínimo",IF(E15=F15,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="16">
@@ -901,15 +901,15 @@
       </c>
       <c r="G16" s="9">
         <f>MAX(F16-E16,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H16" s="10">
         <f>MAX(G16,ROUND(F16*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I16" s="6">
+        <v>2</v>
+      </c>
+      <c r="I16" s="6" t="str">
         <f>IF(E16&lt;=0,"Crítico",IF(E16&lt;F16,"Abaixo do Mínimo",IF(E16=F16,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="17">
@@ -933,15 +933,15 @@
       </c>
       <c r="G17" s="9">
         <f>MAX(F17-E17,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H17" s="10">
         <f>MAX(G17,ROUND(F17*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I17" s="6">
+        <v>1</v>
+      </c>
+      <c r="I17" s="6" t="str">
         <f>IF(E17&lt;=0,"Crítico",IF(E17&lt;F17,"Abaixo do Mínimo",IF(E17=F17,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="18">
@@ -965,15 +965,15 @@
       </c>
       <c r="G18" s="9">
         <f>MAX(F18-E18,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H18" s="10">
         <f>MAX(G18,ROUND(F18*$C$5,0))</f>
-        <v/>
-      </c>
-      <c r="I18" s="6">
+        <v>1</v>
+      </c>
+      <c r="I18" s="6" t="str">
         <f>IF(E18&lt;=0,"Crítico",IF(E18&lt;F18,"Abaixo do Mínimo",IF(E18=F18,"No Mínimo","Ok")))</f>
-        <v/>
+        <v>No Mínimo</v>
       </c>
     </row>
     <row r="19">
@@ -983,20 +983,20 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="12" t="str">
         <f>COUNTA(B9:B18)&amp;" itens"</f>
-        <v/>
+        <v>10 itens</v>
       </c>
       <c r="D19" s="11" t="n"/>
       <c r="E19" s="11" t="n"/>
       <c r="F19" s="11" t="n"/>
       <c r="G19" s="13">
         <f>SUM(G9:G18)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H19" s="13">
         <f>SUM(H9:H18)</f>
-        <v/>
+        <v>280</v>
       </c>
       <c r="I19" s="11" t="n"/>
     </row>
@@ -1064,7 +1064,7 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>